<commit_message>
Fill partner tracker from Foundry solution catalog
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XQ6kcbnMZ7aS7w41Q1Bb6Y
</commit_message>
<xml_diff>
--- a/exports/ke-hoach-partnership-google-sheet.xlsx
+++ b/exports/ke-hoach-partnership-google-sheet.xlsx
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Sổ đối tác toàn công ty'!$A$4:$J$34</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Theo dõi partner'!$A$4:$O$105</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Theo dõi partner'!$A$4:$O$104</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'V-Tech Hub'!$A$4:$L$24</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="219">
   <si>
     <t xml:space="preserve">Kế hoạch phòng Partnership: tổng quan</t>
   </si>
@@ -164,10 +164,10 @@
     <t xml:space="preserve">2. Sheet V-Tech Hub: cập nhật Trạng thái và Ngày hoàn thành mỗi khi xong việc; có thể sửa số ngày hạn.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Sheet Theo dõi partner: mỗi partner một dòng, cập nhật Bước hiện tại và Việc tiếp theo; dòng 5 là dòng ví dụ, xóa khi nhập.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Sheet Sổ đối tác toàn công ty: điền dần khi xác nhận hợp đồng; sáu dòng đầu lấy từ tên nêu trên trang Foundry, chưa xác nhận.</t>
+    <t xml:space="preserve">3. Sheet Theo dõi partner: mỗi partner một dòng; ba dòng đầu lấy từ file danh mục solution, cập nhật Bước hiện tại, Hạng và Việc tiếp theo khi có tiến triển.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Sheet Sổ đối tác toàn công ty: điền dần khi xác nhận hợp đồng; ba hãng công nghệ lấy từ file danh mục, bốn đối tác hạ tầng lấy từ trang Foundry, chưa xác nhận.</t>
   </si>
   <si>
     <t xml:space="preserve">5. Sheet Nhịp làm việc: ghi ngày làm lần gần nhất để biết khi nào đến hạn lần sau.</t>
@@ -488,7 +488,7 @@
     <t xml:space="preserve">Theo dõi partner (mỗi partner một dòng)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dòng 5 là dòng ví dụ (chữ xám nghiêng), xóa hoặc ghi đè khi bắt đầu nhập. Dòng 6 trở đi là dữ liệu thật. Chọn loại, ngành, bước và hạng từ danh sách thả xuống. Cột Cảnh báo tự báo quá hạn việc tiếp theo hoặc hơn 30 ngày chưa liên hệ.</t>
+    <t xml:space="preserve">Ba dòng đầu lấy từ file Vtech_Foundry_Danh_muc_Solutions_Chi_tiet.xlsx (danh mục solution). Ngành, giải pháp, việc tiếp theo và ghi chú lấy từ file đó; các ô còn trống (đầu mối, điểm phù hợp, hạng, ngày liên hệ) bạn tự điền. Chọn loại, bước và hạng từ danh sách thả xuống; cột Ngành cho phép nhập nhiều ngành, cách nhau bằng dấu chấm phẩy. Cột Cảnh báo tự báo quá hạn việc tiếp theo hoặc hơn 30 ngày chưa liên hệ.</t>
   </si>
   <si>
     <t xml:space="preserve">Tên partner</t>
@@ -527,34 +527,58 @@
     <t xml:space="preserve">Hạn việc tiếp theo</t>
   </si>
   <si>
-    <t xml:space="preserve">(Ví dụ) Công ty ABC</t>
+    <t xml:space="preserve">SearchInform</t>
   </si>
   <si>
     <t xml:space="preserve">A. Technology</t>
   </si>
   <si>
-    <t xml:space="preserve">BFSI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data Loss Prevention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tên và số điện thoại</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tên bạn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gửi hồ sơ năng lực cho Presales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dòng ví dụ, xóa khi bắt đầu nhập</t>
+    <t xml:space="preserve">BFSI; Y tế; Sản xuất; Chính phủ; Bán lẻ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SearchInform DLP (Data Loss Prevention)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xác minh quyền phân phối, module và phạm vi triển khai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trạng thái thương mại: Cần xác minh. Chưa chứng minh đã ký hợp đồng phân phối (theo sheet Tong quan của file danh mục). Nguồn: Solution Master / trang sản phẩm SearchInform. Chuyên gia trên trang Foundry: Hoàng Tuấn Anh (Country Director).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DatumBridge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BFSI; Chính phủ; Bán lẻ (và Enterprise, Services, Finance)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI Legal &amp; Compliance; AI SuperSales &amp; Assistant; Debt Collection AI Agent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xác minh nguồn dữ liệu, giới hạn, tích hợp và quyền công bố; riêng Debt Collection: tuân thủ pháp lý và giới hạn tự động hóa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trạng thái thương mại: Cần xác minh. Chưa chứng minh đã ký hợp đồng phân phối (theo sheet Tong quan của file danh mục). Nguồn: Solution Master / thông tin DatumBridge đã trao đổi. 3 giải pháp. Chuyên gia trên trang Foundry: Nguyễn Đức Anh (Founder và CEO).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lumination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giáo dục; Y tế</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI Admissions CRM; AI Healthcare &amp; Insurance Assistant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xác minh phạm vi CRM và AI, tích hợp, bảo mật dữ liệu y tế và phạm vi sử dụng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trạng thái thương mại: Cần xác minh. Chưa chứng minh đã ký hợp đồng phân phối (theo sheet Tong quan của file danh mục). Nguồn: Solution Master / thông tin Lumination đã trao đổi. 2 giải pháp.</t>
   </si>
   <si>
     <t xml:space="preserve">Sổ quan hệ đối tác toàn công ty</t>
   </si>
   <si>
-    <t xml:space="preserve">Ai đang hợp tác với VNETWORK, đã ký gì, ai phụ trách, còn hiệu lực không. Sáu dòng đầu lấy từ tên được nêu trên trang V-Tech Foundry; loại thỏa thuận và quyền dùng tên đều ghi "Chưa rõ" cho đến khi xác nhận bằng văn bản. Cột Tình trạng tự tính từ ngày hết hạn (sắp hết hạn = còn dưới 60 ngày).</t>
+    <t xml:space="preserve">Ai đang hợp tác với VNETWORK, đã ký gì, ai phụ trách, còn hiệu lực không. Ba dòng đầu (SearchInform, DatumBridge, Lumination) lấy từ file danh mục solution; bốn dòng hạ tầng lấy từ tên được nêu trên trang V-Tech Foundry. Loại thỏa thuận và quyền dùng tên đều ghi "Chưa rõ" cho đến khi xác nhận bằng văn bản. Cột Tình trạng tự tính từ ngày hết hạn (sắp hết hạn = còn dưới 60 ngày).</t>
   </si>
   <si>
     <t xml:space="preserve">Tên đối tác</t>
@@ -587,6 +611,18 @@
     <t xml:space="preserve">Nguồn và ghi chú</t>
   </si>
   <si>
+    <t xml:space="preserve">Hãng công nghệ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Có trong file danh mục solution, trạng thái thương mại cần xác minh; chưa chứng minh đã ký hợp đồng phân phối (1 giải pháp: DLP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Có trong file danh mục solution, trạng thái thương mại cần xác minh; chưa chứng minh đã ký hợp đồng phân phối (3 giải pháp AI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Có trong file danh mục solution, trạng thái thương mại cần xác minh; chưa chứng minh đã ký hợp đồng phân phối (2 giải pháp AI)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Viettel IDC</t>
   </si>
   <si>
@@ -603,18 +639,6 @@
   </si>
   <si>
     <t xml:space="preserve">Mobifone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DatumBridge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hãng công nghệ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Có chuyên gia trên trang Foundry, cần xác nhận quan hệ hợp tác</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SearchInform</t>
   </si>
   <si>
     <t xml:space="preserve">Nhịp làm việc định kỳ</t>
@@ -675,7 +699,7 @@
     <numFmt numFmtId="166" formatCode="General"/>
     <numFmt numFmtId="167" formatCode="0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -730,14 +754,6 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -824,7 +840,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -905,14 +921,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -926,7 +934,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="9">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -997,14 +1005,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF7F7F7F"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <colors>
     <indexedColors>
@@ -1023,7 +1023,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF7F7F7F"/>
+      <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
@@ -1463,14 +1463,14 @@
         <v>23</v>
       </c>
       <c r="B16" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$H$6:$H$105,A16)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$H$5:$H$104,A16)</f>
         <v>0</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$I$6:$I$105,D16)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$I$5:$I$104,D16)</f>
         <v>0</v>
       </c>
     </row>
@@ -1479,14 +1479,14 @@
         <v>25</v>
       </c>
       <c r="B17" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$H$6:$H$105,A17)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$H$5:$H$104,A17)</f>
         <v>0</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>26</v>
       </c>
       <c r="E17" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$I$6:$I$105,D17)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$I$5:$I$104,D17)</f>
         <v>0</v>
       </c>
     </row>
@@ -1495,14 +1495,14 @@
         <v>27</v>
       </c>
       <c r="B18" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$H$6:$H$105,A18)</f>
-        <v>0</v>
+        <f aca="false">COUNTIF('Theo dõi partner'!$H$5:$H$104,A18)</f>
+        <v>3</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>28</v>
       </c>
       <c r="E18" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$I$6:$I$105,D18)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$I$5:$I$104,D18)</f>
         <v>0</v>
       </c>
     </row>
@@ -1511,14 +1511,14 @@
         <v>29</v>
       </c>
       <c r="B19" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$H$6:$H$105,A19)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$H$5:$H$104,A19)</f>
         <v>0</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>30</v>
       </c>
       <c r="E19" s="10" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$N$6:$N$105,"?*")</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$N$5:$N$104,"?*")</f>
         <v>0</v>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
         <v>31</v>
       </c>
       <c r="B20" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$H$6:$H$105,A20)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$H$5:$H$104,A20)</f>
         <v>0</v>
       </c>
     </row>
@@ -1536,7 +1536,7 @@
         <v>32</v>
       </c>
       <c r="B21" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$H$6:$H$105,A21)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$H$5:$H$104,A21)</f>
         <v>0</v>
       </c>
       <c r="D21" s="5" t="s">
@@ -1551,7 +1551,7 @@
         <v>35</v>
       </c>
       <c r="B22" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$H$6:$H$105,A22)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$H$5:$H$104,A22)</f>
         <v>0</v>
       </c>
       <c r="D22" s="6" t="s">
@@ -1567,7 +1567,7 @@
         <v>37</v>
       </c>
       <c r="B23" s="7" t="n">
-        <f aca="false">COUNTIF('Theo dõi partner'!$H$6:$H$105,A23)</f>
+        <f aca="false">COUNTIF('Theo dõi partner'!$H$5:$H$104,A23)</f>
         <v>0</v>
       </c>
       <c r="D23" s="6" t="s">
@@ -1583,8 +1583,8 @@
         <v>39</v>
       </c>
       <c r="B24" s="10" t="n">
-        <f aca="false">COUNTA('Theo dõi partner'!$B$6:$B$105)</f>
-        <v>0</v>
+        <f aca="false">COUNTA('Theo dõi partner'!$B$5:$B$104)</f>
+        <v>3</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>40</v>
@@ -2701,7 +2701,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O105"/>
+  <dimension ref="A1:O104"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2789,96 +2789,117 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20"/>
-      <c r="B5" s="20" t="s">
+    <row r="5" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="M5" s="17"/>
+      <c r="N5" s="20" t="str">
+        <f aca="true">IF(B5="","",IF(AND(M5&lt;&gt;"",M5&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K5&lt;&gt;"",TODAY()-K5&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
+        <v/>
+      </c>
+      <c r="O5" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" s="21" t="n">
-        <v>46328</v>
-      </c>
-      <c r="L5" s="20" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="M5" s="21" t="n">
-        <v>46335</v>
-      </c>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20" t="s">
+      <c r="C6" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="D6" s="19" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
+      <c r="E6" s="19" t="s">
+        <v>173</v>
+      </c>
       <c r="F6" s="19"/>
       <c r="G6" s="19"/>
-      <c r="H6" s="15"/>
+      <c r="H6" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="I6" s="15"/>
       <c r="J6" s="15"/>
       <c r="K6" s="17"/>
-      <c r="L6" s="19"/>
+      <c r="L6" s="19" t="s">
+        <v>174</v>
+      </c>
       <c r="M6" s="17"/>
-      <c r="N6" s="22" t="str">
+      <c r="N6" s="20" t="str">
         <f aca="true">IF(B6="","",IF(AND(M6&lt;&gt;"",M6&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K6&lt;&gt;"",TODAY()-K6&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
-      <c r="O6" s="19"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O6" s="19" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
+        <v>3</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>178</v>
+      </c>
       <c r="F7" s="19"/>
       <c r="G7" s="19"/>
-      <c r="H7" s="15"/>
+      <c r="H7" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="I7" s="15"/>
       <c r="J7" s="15"/>
       <c r="K7" s="17"/>
-      <c r="L7" s="19"/>
+      <c r="L7" s="19" t="s">
+        <v>179</v>
+      </c>
       <c r="M7" s="17"/>
-      <c r="N7" s="22" t="str">
+      <c r="N7" s="20" t="str">
         <f aca="true">IF(B7="","",IF(AND(M7&lt;&gt;"",M7&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K7&lt;&gt;"",TODAY()-K7&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
-      <c r="O7" s="19"/>
+      <c r="O7" s="19" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="15"/>
@@ -2892,7 +2913,7 @@
       <c r="K8" s="17"/>
       <c r="L8" s="19"/>
       <c r="M8" s="17"/>
-      <c r="N8" s="22" t="str">
+      <c r="N8" s="20" t="str">
         <f aca="true">IF(B8="","",IF(AND(M8&lt;&gt;"",M8&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K8&lt;&gt;"",TODAY()-K8&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -2900,7 +2921,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" s="19"/>
       <c r="C9" s="15"/>
@@ -2914,7 +2935,7 @@
       <c r="K9" s="17"/>
       <c r="L9" s="19"/>
       <c r="M9" s="17"/>
-      <c r="N9" s="22" t="str">
+      <c r="N9" s="20" t="str">
         <f aca="true">IF(B9="","",IF(AND(M9&lt;&gt;"",M9&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K9&lt;&gt;"",TODAY()-K9&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -2922,7 +2943,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" s="19"/>
       <c r="C10" s="15"/>
@@ -2936,7 +2957,7 @@
       <c r="K10" s="17"/>
       <c r="L10" s="19"/>
       <c r="M10" s="17"/>
-      <c r="N10" s="22" t="str">
+      <c r="N10" s="20" t="str">
         <f aca="true">IF(B10="","",IF(AND(M10&lt;&gt;"",M10&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K10&lt;&gt;"",TODAY()-K10&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -2944,7 +2965,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="15"/>
@@ -2958,7 +2979,7 @@
       <c r="K11" s="17"/>
       <c r="L11" s="19"/>
       <c r="M11" s="17"/>
-      <c r="N11" s="22" t="str">
+      <c r="N11" s="20" t="str">
         <f aca="true">IF(B11="","",IF(AND(M11&lt;&gt;"",M11&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K11&lt;&gt;"",TODAY()-K11&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -2966,7 +2987,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" s="19"/>
       <c r="C12" s="15"/>
@@ -2980,7 +3001,7 @@
       <c r="K12" s="17"/>
       <c r="L12" s="19"/>
       <c r="M12" s="17"/>
-      <c r="N12" s="22" t="str">
+      <c r="N12" s="20" t="str">
         <f aca="true">IF(B12="","",IF(AND(M12&lt;&gt;"",M12&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K12&lt;&gt;"",TODAY()-K12&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -2988,7 +3009,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B13" s="19"/>
       <c r="C13" s="15"/>
@@ -3002,7 +3023,7 @@
       <c r="K13" s="17"/>
       <c r="L13" s="19"/>
       <c r="M13" s="17"/>
-      <c r="N13" s="22" t="str">
+      <c r="N13" s="20" t="str">
         <f aca="true">IF(B13="","",IF(AND(M13&lt;&gt;"",M13&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K13&lt;&gt;"",TODAY()-K13&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3010,7 +3031,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B14" s="19"/>
       <c r="C14" s="15"/>
@@ -3024,7 +3045,7 @@
       <c r="K14" s="17"/>
       <c r="L14" s="19"/>
       <c r="M14" s="17"/>
-      <c r="N14" s="22" t="str">
+      <c r="N14" s="20" t="str">
         <f aca="true">IF(B14="","",IF(AND(M14&lt;&gt;"",M14&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K14&lt;&gt;"",TODAY()-K14&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3032,7 +3053,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B15" s="19"/>
       <c r="C15" s="15"/>
@@ -3046,7 +3067,7 @@
       <c r="K15" s="17"/>
       <c r="L15" s="19"/>
       <c r="M15" s="17"/>
-      <c r="N15" s="22" t="str">
+      <c r="N15" s="20" t="str">
         <f aca="true">IF(B15="","",IF(AND(M15&lt;&gt;"",M15&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K15&lt;&gt;"",TODAY()-K15&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3054,7 +3075,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16" s="19"/>
       <c r="C16" s="15"/>
@@ -3068,7 +3089,7 @@
       <c r="K16" s="17"/>
       <c r="L16" s="19"/>
       <c r="M16" s="17"/>
-      <c r="N16" s="22" t="str">
+      <c r="N16" s="20" t="str">
         <f aca="true">IF(B16="","",IF(AND(M16&lt;&gt;"",M16&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K16&lt;&gt;"",TODAY()-K16&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3076,7 +3097,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="15"/>
@@ -3090,7 +3111,7 @@
       <c r="K17" s="17"/>
       <c r="L17" s="19"/>
       <c r="M17" s="17"/>
-      <c r="N17" s="22" t="str">
+      <c r="N17" s="20" t="str">
         <f aca="true">IF(B17="","",IF(AND(M17&lt;&gt;"",M17&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K17&lt;&gt;"",TODAY()-K17&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3098,7 +3119,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B18" s="19"/>
       <c r="C18" s="15"/>
@@ -3112,7 +3133,7 @@
       <c r="K18" s="17"/>
       <c r="L18" s="19"/>
       <c r="M18" s="17"/>
-      <c r="N18" s="22" t="str">
+      <c r="N18" s="20" t="str">
         <f aca="true">IF(B18="","",IF(AND(M18&lt;&gt;"",M18&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K18&lt;&gt;"",TODAY()-K18&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3120,7 +3141,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="15"/>
@@ -3134,7 +3155,7 @@
       <c r="K19" s="17"/>
       <c r="L19" s="19"/>
       <c r="M19" s="17"/>
-      <c r="N19" s="22" t="str">
+      <c r="N19" s="20" t="str">
         <f aca="true">IF(B19="","",IF(AND(M19&lt;&gt;"",M19&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K19&lt;&gt;"",TODAY()-K19&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3142,7 +3163,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B20" s="19"/>
       <c r="C20" s="15"/>
@@ -3156,7 +3177,7 @@
       <c r="K20" s="17"/>
       <c r="L20" s="19"/>
       <c r="M20" s="17"/>
-      <c r="N20" s="22" t="str">
+      <c r="N20" s="20" t="str">
         <f aca="true">IF(B20="","",IF(AND(M20&lt;&gt;"",M20&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K20&lt;&gt;"",TODAY()-K20&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3164,7 +3185,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="15"/>
@@ -3178,7 +3199,7 @@
       <c r="K21" s="17"/>
       <c r="L21" s="19"/>
       <c r="M21" s="17"/>
-      <c r="N21" s="22" t="str">
+      <c r="N21" s="20" t="str">
         <f aca="true">IF(B21="","",IF(AND(M21&lt;&gt;"",M21&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K21&lt;&gt;"",TODAY()-K21&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3186,7 +3207,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B22" s="19"/>
       <c r="C22" s="15"/>
@@ -3200,7 +3221,7 @@
       <c r="K22" s="17"/>
       <c r="L22" s="19"/>
       <c r="M22" s="17"/>
-      <c r="N22" s="22" t="str">
+      <c r="N22" s="20" t="str">
         <f aca="true">IF(B22="","",IF(AND(M22&lt;&gt;"",M22&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K22&lt;&gt;"",TODAY()-K22&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3208,7 +3229,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="15"/>
@@ -3222,7 +3243,7 @@
       <c r="K23" s="17"/>
       <c r="L23" s="19"/>
       <c r="M23" s="17"/>
-      <c r="N23" s="22" t="str">
+      <c r="N23" s="20" t="str">
         <f aca="true">IF(B23="","",IF(AND(M23&lt;&gt;"",M23&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K23&lt;&gt;"",TODAY()-K23&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3230,7 +3251,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="15"/>
@@ -3244,7 +3265,7 @@
       <c r="K24" s="17"/>
       <c r="L24" s="19"/>
       <c r="M24" s="17"/>
-      <c r="N24" s="22" t="str">
+      <c r="N24" s="20" t="str">
         <f aca="true">IF(B24="","",IF(AND(M24&lt;&gt;"",M24&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K24&lt;&gt;"",TODAY()-K24&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3252,7 +3273,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B25" s="19"/>
       <c r="C25" s="15"/>
@@ -3266,7 +3287,7 @@
       <c r="K25" s="17"/>
       <c r="L25" s="19"/>
       <c r="M25" s="17"/>
-      <c r="N25" s="22" t="str">
+      <c r="N25" s="20" t="str">
         <f aca="true">IF(B25="","",IF(AND(M25&lt;&gt;"",M25&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K25&lt;&gt;"",TODAY()-K25&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3274,7 +3295,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B26" s="19"/>
       <c r="C26" s="15"/>
@@ -3288,7 +3309,7 @@
       <c r="K26" s="17"/>
       <c r="L26" s="19"/>
       <c r="M26" s="17"/>
-      <c r="N26" s="22" t="str">
+      <c r="N26" s="20" t="str">
         <f aca="true">IF(B26="","",IF(AND(M26&lt;&gt;"",M26&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K26&lt;&gt;"",TODAY()-K26&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3296,7 +3317,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B27" s="19"/>
       <c r="C27" s="15"/>
@@ -3310,7 +3331,7 @@
       <c r="K27" s="17"/>
       <c r="L27" s="19"/>
       <c r="M27" s="17"/>
-      <c r="N27" s="22" t="str">
+      <c r="N27" s="20" t="str">
         <f aca="true">IF(B27="","",IF(AND(M27&lt;&gt;"",M27&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K27&lt;&gt;"",TODAY()-K27&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3318,7 +3339,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="15"/>
@@ -3332,7 +3353,7 @@
       <c r="K28" s="17"/>
       <c r="L28" s="19"/>
       <c r="M28" s="17"/>
-      <c r="N28" s="22" t="str">
+      <c r="N28" s="20" t="str">
         <f aca="true">IF(B28="","",IF(AND(M28&lt;&gt;"",M28&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K28&lt;&gt;"",TODAY()-K28&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3340,7 +3361,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B29" s="19"/>
       <c r="C29" s="15"/>
@@ -3354,7 +3375,7 @@
       <c r="K29" s="17"/>
       <c r="L29" s="19"/>
       <c r="M29" s="17"/>
-      <c r="N29" s="22" t="str">
+      <c r="N29" s="20" t="str">
         <f aca="true">IF(B29="","",IF(AND(M29&lt;&gt;"",M29&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K29&lt;&gt;"",TODAY()-K29&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3362,7 +3383,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B30" s="19"/>
       <c r="C30" s="15"/>
@@ -3376,7 +3397,7 @@
       <c r="K30" s="17"/>
       <c r="L30" s="19"/>
       <c r="M30" s="17"/>
-      <c r="N30" s="22" t="str">
+      <c r="N30" s="20" t="str">
         <f aca="true">IF(B30="","",IF(AND(M30&lt;&gt;"",M30&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K30&lt;&gt;"",TODAY()-K30&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3384,7 +3405,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B31" s="19"/>
       <c r="C31" s="15"/>
@@ -3398,7 +3419,7 @@
       <c r="K31" s="17"/>
       <c r="L31" s="19"/>
       <c r="M31" s="17"/>
-      <c r="N31" s="22" t="str">
+      <c r="N31" s="20" t="str">
         <f aca="true">IF(B31="","",IF(AND(M31&lt;&gt;"",M31&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K31&lt;&gt;"",TODAY()-K31&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3406,7 +3427,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B32" s="19"/>
       <c r="C32" s="15"/>
@@ -3420,7 +3441,7 @@
       <c r="K32" s="17"/>
       <c r="L32" s="19"/>
       <c r="M32" s="17"/>
-      <c r="N32" s="22" t="str">
+      <c r="N32" s="20" t="str">
         <f aca="true">IF(B32="","",IF(AND(M32&lt;&gt;"",M32&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K32&lt;&gt;"",TODAY()-K32&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3428,7 +3449,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B33" s="19"/>
       <c r="C33" s="15"/>
@@ -3442,7 +3463,7 @@
       <c r="K33" s="17"/>
       <c r="L33" s="19"/>
       <c r="M33" s="17"/>
-      <c r="N33" s="22" t="str">
+      <c r="N33" s="20" t="str">
         <f aca="true">IF(B33="","",IF(AND(M33&lt;&gt;"",M33&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K33&lt;&gt;"",TODAY()-K33&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3450,7 +3471,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B34" s="19"/>
       <c r="C34" s="15"/>
@@ -3464,7 +3485,7 @@
       <c r="K34" s="17"/>
       <c r="L34" s="19"/>
       <c r="M34" s="17"/>
-      <c r="N34" s="22" t="str">
+      <c r="N34" s="20" t="str">
         <f aca="true">IF(B34="","",IF(AND(M34&lt;&gt;"",M34&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K34&lt;&gt;"",TODAY()-K34&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3472,7 +3493,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B35" s="19"/>
       <c r="C35" s="15"/>
@@ -3486,7 +3507,7 @@
       <c r="K35" s="17"/>
       <c r="L35" s="19"/>
       <c r="M35" s="17"/>
-      <c r="N35" s="22" t="str">
+      <c r="N35" s="20" t="str">
         <f aca="true">IF(B35="","",IF(AND(M35&lt;&gt;"",M35&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K35&lt;&gt;"",TODAY()-K35&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3494,7 +3515,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B36" s="19"/>
       <c r="C36" s="15"/>
@@ -3508,7 +3529,7 @@
       <c r="K36" s="17"/>
       <c r="L36" s="19"/>
       <c r="M36" s="17"/>
-      <c r="N36" s="22" t="str">
+      <c r="N36" s="20" t="str">
         <f aca="true">IF(B36="","",IF(AND(M36&lt;&gt;"",M36&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K36&lt;&gt;"",TODAY()-K36&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3516,7 +3537,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B37" s="19"/>
       <c r="C37" s="15"/>
@@ -3530,7 +3551,7 @@
       <c r="K37" s="17"/>
       <c r="L37" s="19"/>
       <c r="M37" s="17"/>
-      <c r="N37" s="22" t="str">
+      <c r="N37" s="20" t="str">
         <f aca="true">IF(B37="","",IF(AND(M37&lt;&gt;"",M37&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K37&lt;&gt;"",TODAY()-K37&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3538,7 +3559,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B38" s="19"/>
       <c r="C38" s="15"/>
@@ -3552,7 +3573,7 @@
       <c r="K38" s="17"/>
       <c r="L38" s="19"/>
       <c r="M38" s="17"/>
-      <c r="N38" s="22" t="str">
+      <c r="N38" s="20" t="str">
         <f aca="true">IF(B38="","",IF(AND(M38&lt;&gt;"",M38&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K38&lt;&gt;"",TODAY()-K38&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3560,7 +3581,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B39" s="19"/>
       <c r="C39" s="15"/>
@@ -3574,7 +3595,7 @@
       <c r="K39" s="17"/>
       <c r="L39" s="19"/>
       <c r="M39" s="17"/>
-      <c r="N39" s="22" t="str">
+      <c r="N39" s="20" t="str">
         <f aca="true">IF(B39="","",IF(AND(M39&lt;&gt;"",M39&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K39&lt;&gt;"",TODAY()-K39&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3582,7 +3603,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B40" s="19"/>
       <c r="C40" s="15"/>
@@ -3596,7 +3617,7 @@
       <c r="K40" s="17"/>
       <c r="L40" s="19"/>
       <c r="M40" s="17"/>
-      <c r="N40" s="22" t="str">
+      <c r="N40" s="20" t="str">
         <f aca="true">IF(B40="","",IF(AND(M40&lt;&gt;"",M40&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K40&lt;&gt;"",TODAY()-K40&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3604,7 +3625,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B41" s="19"/>
       <c r="C41" s="15"/>
@@ -3618,7 +3639,7 @@
       <c r="K41" s="17"/>
       <c r="L41" s="19"/>
       <c r="M41" s="17"/>
-      <c r="N41" s="22" t="str">
+      <c r="N41" s="20" t="str">
         <f aca="true">IF(B41="","",IF(AND(M41&lt;&gt;"",M41&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K41&lt;&gt;"",TODAY()-K41&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3626,7 +3647,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B42" s="19"/>
       <c r="C42" s="15"/>
@@ -3640,7 +3661,7 @@
       <c r="K42" s="17"/>
       <c r="L42" s="19"/>
       <c r="M42" s="17"/>
-      <c r="N42" s="22" t="str">
+      <c r="N42" s="20" t="str">
         <f aca="true">IF(B42="","",IF(AND(M42&lt;&gt;"",M42&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K42&lt;&gt;"",TODAY()-K42&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3648,7 +3669,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B43" s="19"/>
       <c r="C43" s="15"/>
@@ -3662,7 +3683,7 @@
       <c r="K43" s="17"/>
       <c r="L43" s="19"/>
       <c r="M43" s="17"/>
-      <c r="N43" s="22" t="str">
+      <c r="N43" s="20" t="str">
         <f aca="true">IF(B43="","",IF(AND(M43&lt;&gt;"",M43&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K43&lt;&gt;"",TODAY()-K43&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3670,7 +3691,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B44" s="19"/>
       <c r="C44" s="15"/>
@@ -3684,7 +3705,7 @@
       <c r="K44" s="17"/>
       <c r="L44" s="19"/>
       <c r="M44" s="17"/>
-      <c r="N44" s="22" t="str">
+      <c r="N44" s="20" t="str">
         <f aca="true">IF(B44="","",IF(AND(M44&lt;&gt;"",M44&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K44&lt;&gt;"",TODAY()-K44&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3692,7 +3713,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B45" s="19"/>
       <c r="C45" s="15"/>
@@ -3706,7 +3727,7 @@
       <c r="K45" s="17"/>
       <c r="L45" s="19"/>
       <c r="M45" s="17"/>
-      <c r="N45" s="22" t="str">
+      <c r="N45" s="20" t="str">
         <f aca="true">IF(B45="","",IF(AND(M45&lt;&gt;"",M45&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K45&lt;&gt;"",TODAY()-K45&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3714,7 +3735,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B46" s="19"/>
       <c r="C46" s="15"/>
@@ -3728,7 +3749,7 @@
       <c r="K46" s="17"/>
       <c r="L46" s="19"/>
       <c r="M46" s="17"/>
-      <c r="N46" s="22" t="str">
+      <c r="N46" s="20" t="str">
         <f aca="true">IF(B46="","",IF(AND(M46&lt;&gt;"",M46&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K46&lt;&gt;"",TODAY()-K46&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3736,7 +3757,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B47" s="19"/>
       <c r="C47" s="15"/>
@@ -3750,7 +3771,7 @@
       <c r="K47" s="17"/>
       <c r="L47" s="19"/>
       <c r="M47" s="17"/>
-      <c r="N47" s="22" t="str">
+      <c r="N47" s="20" t="str">
         <f aca="true">IF(B47="","",IF(AND(M47&lt;&gt;"",M47&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K47&lt;&gt;"",TODAY()-K47&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3758,7 +3779,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B48" s="19"/>
       <c r="C48" s="15"/>
@@ -3772,7 +3793,7 @@
       <c r="K48" s="17"/>
       <c r="L48" s="19"/>
       <c r="M48" s="17"/>
-      <c r="N48" s="22" t="str">
+      <c r="N48" s="20" t="str">
         <f aca="true">IF(B48="","",IF(AND(M48&lt;&gt;"",M48&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K48&lt;&gt;"",TODAY()-K48&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3780,7 +3801,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B49" s="19"/>
       <c r="C49" s="15"/>
@@ -3794,7 +3815,7 @@
       <c r="K49" s="17"/>
       <c r="L49" s="19"/>
       <c r="M49" s="17"/>
-      <c r="N49" s="22" t="str">
+      <c r="N49" s="20" t="str">
         <f aca="true">IF(B49="","",IF(AND(M49&lt;&gt;"",M49&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K49&lt;&gt;"",TODAY()-K49&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3802,7 +3823,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B50" s="19"/>
       <c r="C50" s="15"/>
@@ -3816,7 +3837,7 @@
       <c r="K50" s="17"/>
       <c r="L50" s="19"/>
       <c r="M50" s="17"/>
-      <c r="N50" s="22" t="str">
+      <c r="N50" s="20" t="str">
         <f aca="true">IF(B50="","",IF(AND(M50&lt;&gt;"",M50&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K50&lt;&gt;"",TODAY()-K50&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3824,7 +3845,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B51" s="19"/>
       <c r="C51" s="15"/>
@@ -3838,7 +3859,7 @@
       <c r="K51" s="17"/>
       <c r="L51" s="19"/>
       <c r="M51" s="17"/>
-      <c r="N51" s="22" t="str">
+      <c r="N51" s="20" t="str">
         <f aca="true">IF(B51="","",IF(AND(M51&lt;&gt;"",M51&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K51&lt;&gt;"",TODAY()-K51&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3846,7 +3867,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B52" s="19"/>
       <c r="C52" s="15"/>
@@ -3860,7 +3881,7 @@
       <c r="K52" s="17"/>
       <c r="L52" s="19"/>
       <c r="M52" s="17"/>
-      <c r="N52" s="22" t="str">
+      <c r="N52" s="20" t="str">
         <f aca="true">IF(B52="","",IF(AND(M52&lt;&gt;"",M52&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K52&lt;&gt;"",TODAY()-K52&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3868,7 +3889,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B53" s="19"/>
       <c r="C53" s="15"/>
@@ -3882,7 +3903,7 @@
       <c r="K53" s="17"/>
       <c r="L53" s="19"/>
       <c r="M53" s="17"/>
-      <c r="N53" s="22" t="str">
+      <c r="N53" s="20" t="str">
         <f aca="true">IF(B53="","",IF(AND(M53&lt;&gt;"",M53&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K53&lt;&gt;"",TODAY()-K53&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3890,7 +3911,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B54" s="19"/>
       <c r="C54" s="15"/>
@@ -3904,7 +3925,7 @@
       <c r="K54" s="17"/>
       <c r="L54" s="19"/>
       <c r="M54" s="17"/>
-      <c r="N54" s="22" t="str">
+      <c r="N54" s="20" t="str">
         <f aca="true">IF(B54="","",IF(AND(M54&lt;&gt;"",M54&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K54&lt;&gt;"",TODAY()-K54&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3912,7 +3933,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B55" s="19"/>
       <c r="C55" s="15"/>
@@ -3926,7 +3947,7 @@
       <c r="K55" s="17"/>
       <c r="L55" s="19"/>
       <c r="M55" s="17"/>
-      <c r="N55" s="22" t="str">
+      <c r="N55" s="20" t="str">
         <f aca="true">IF(B55="","",IF(AND(M55&lt;&gt;"",M55&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K55&lt;&gt;"",TODAY()-K55&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3934,7 +3955,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B56" s="19"/>
       <c r="C56" s="15"/>
@@ -3948,7 +3969,7 @@
       <c r="K56" s="17"/>
       <c r="L56" s="19"/>
       <c r="M56" s="17"/>
-      <c r="N56" s="22" t="str">
+      <c r="N56" s="20" t="str">
         <f aca="true">IF(B56="","",IF(AND(M56&lt;&gt;"",M56&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K56&lt;&gt;"",TODAY()-K56&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3956,7 +3977,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B57" s="19"/>
       <c r="C57" s="15"/>
@@ -3970,7 +3991,7 @@
       <c r="K57" s="17"/>
       <c r="L57" s="19"/>
       <c r="M57" s="17"/>
-      <c r="N57" s="22" t="str">
+      <c r="N57" s="20" t="str">
         <f aca="true">IF(B57="","",IF(AND(M57&lt;&gt;"",M57&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K57&lt;&gt;"",TODAY()-K57&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -3978,7 +3999,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B58" s="19"/>
       <c r="C58" s="15"/>
@@ -3992,7 +4013,7 @@
       <c r="K58" s="17"/>
       <c r="L58" s="19"/>
       <c r="M58" s="17"/>
-      <c r="N58" s="22" t="str">
+      <c r="N58" s="20" t="str">
         <f aca="true">IF(B58="","",IF(AND(M58&lt;&gt;"",M58&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K58&lt;&gt;"",TODAY()-K58&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4000,7 +4021,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B59" s="19"/>
       <c r="C59" s="15"/>
@@ -4014,7 +4035,7 @@
       <c r="K59" s="17"/>
       <c r="L59" s="19"/>
       <c r="M59" s="17"/>
-      <c r="N59" s="22" t="str">
+      <c r="N59" s="20" t="str">
         <f aca="true">IF(B59="","",IF(AND(M59&lt;&gt;"",M59&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K59&lt;&gt;"",TODAY()-K59&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4022,7 +4043,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B60" s="19"/>
       <c r="C60" s="15"/>
@@ -4036,7 +4057,7 @@
       <c r="K60" s="17"/>
       <c r="L60" s="19"/>
       <c r="M60" s="17"/>
-      <c r="N60" s="22" t="str">
+      <c r="N60" s="20" t="str">
         <f aca="true">IF(B60="","",IF(AND(M60&lt;&gt;"",M60&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K60&lt;&gt;"",TODAY()-K60&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4044,7 +4065,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B61" s="19"/>
       <c r="C61" s="15"/>
@@ -4058,7 +4079,7 @@
       <c r="K61" s="17"/>
       <c r="L61" s="19"/>
       <c r="M61" s="17"/>
-      <c r="N61" s="22" t="str">
+      <c r="N61" s="20" t="str">
         <f aca="true">IF(B61="","",IF(AND(M61&lt;&gt;"",M61&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K61&lt;&gt;"",TODAY()-K61&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4066,7 +4087,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B62" s="19"/>
       <c r="C62" s="15"/>
@@ -4080,7 +4101,7 @@
       <c r="K62" s="17"/>
       <c r="L62" s="19"/>
       <c r="M62" s="17"/>
-      <c r="N62" s="22" t="str">
+      <c r="N62" s="20" t="str">
         <f aca="true">IF(B62="","",IF(AND(M62&lt;&gt;"",M62&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K62&lt;&gt;"",TODAY()-K62&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4088,7 +4109,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B63" s="19"/>
       <c r="C63" s="15"/>
@@ -4102,7 +4123,7 @@
       <c r="K63" s="17"/>
       <c r="L63" s="19"/>
       <c r="M63" s="17"/>
-      <c r="N63" s="22" t="str">
+      <c r="N63" s="20" t="str">
         <f aca="true">IF(B63="","",IF(AND(M63&lt;&gt;"",M63&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K63&lt;&gt;"",TODAY()-K63&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4110,7 +4131,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B64" s="19"/>
       <c r="C64" s="15"/>
@@ -4124,7 +4145,7 @@
       <c r="K64" s="17"/>
       <c r="L64" s="19"/>
       <c r="M64" s="17"/>
-      <c r="N64" s="22" t="str">
+      <c r="N64" s="20" t="str">
         <f aca="true">IF(B64="","",IF(AND(M64&lt;&gt;"",M64&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K64&lt;&gt;"",TODAY()-K64&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4132,7 +4153,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B65" s="19"/>
       <c r="C65" s="15"/>
@@ -4146,7 +4167,7 @@
       <c r="K65" s="17"/>
       <c r="L65" s="19"/>
       <c r="M65" s="17"/>
-      <c r="N65" s="22" t="str">
+      <c r="N65" s="20" t="str">
         <f aca="true">IF(B65="","",IF(AND(M65&lt;&gt;"",M65&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K65&lt;&gt;"",TODAY()-K65&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4154,7 +4175,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B66" s="19"/>
       <c r="C66" s="15"/>
@@ -4168,7 +4189,7 @@
       <c r="K66" s="17"/>
       <c r="L66" s="19"/>
       <c r="M66" s="17"/>
-      <c r="N66" s="22" t="str">
+      <c r="N66" s="20" t="str">
         <f aca="true">IF(B66="","",IF(AND(M66&lt;&gt;"",M66&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K66&lt;&gt;"",TODAY()-K66&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4176,7 +4197,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B67" s="19"/>
       <c r="C67" s="15"/>
@@ -4190,7 +4211,7 @@
       <c r="K67" s="17"/>
       <c r="L67" s="19"/>
       <c r="M67" s="17"/>
-      <c r="N67" s="22" t="str">
+      <c r="N67" s="20" t="str">
         <f aca="true">IF(B67="","",IF(AND(M67&lt;&gt;"",M67&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K67&lt;&gt;"",TODAY()-K67&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4198,7 +4219,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B68" s="19"/>
       <c r="C68" s="15"/>
@@ -4212,7 +4233,7 @@
       <c r="K68" s="17"/>
       <c r="L68" s="19"/>
       <c r="M68" s="17"/>
-      <c r="N68" s="22" t="str">
+      <c r="N68" s="20" t="str">
         <f aca="true">IF(B68="","",IF(AND(M68&lt;&gt;"",M68&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K68&lt;&gt;"",TODAY()-K68&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4220,7 +4241,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B69" s="19"/>
       <c r="C69" s="15"/>
@@ -4234,7 +4255,7 @@
       <c r="K69" s="17"/>
       <c r="L69" s="19"/>
       <c r="M69" s="17"/>
-      <c r="N69" s="22" t="str">
+      <c r="N69" s="20" t="str">
         <f aca="true">IF(B69="","",IF(AND(M69&lt;&gt;"",M69&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K69&lt;&gt;"",TODAY()-K69&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4242,7 +4263,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B70" s="19"/>
       <c r="C70" s="15"/>
@@ -4256,7 +4277,7 @@
       <c r="K70" s="17"/>
       <c r="L70" s="19"/>
       <c r="M70" s="17"/>
-      <c r="N70" s="22" t="str">
+      <c r="N70" s="20" t="str">
         <f aca="true">IF(B70="","",IF(AND(M70&lt;&gt;"",M70&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K70&lt;&gt;"",TODAY()-K70&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4264,7 +4285,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B71" s="19"/>
       <c r="C71" s="15"/>
@@ -4278,7 +4299,7 @@
       <c r="K71" s="17"/>
       <c r="L71" s="19"/>
       <c r="M71" s="17"/>
-      <c r="N71" s="22" t="str">
+      <c r="N71" s="20" t="str">
         <f aca="true">IF(B71="","",IF(AND(M71&lt;&gt;"",M71&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K71&lt;&gt;"",TODAY()-K71&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4286,7 +4307,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B72" s="19"/>
       <c r="C72" s="15"/>
@@ -4300,7 +4321,7 @@
       <c r="K72" s="17"/>
       <c r="L72" s="19"/>
       <c r="M72" s="17"/>
-      <c r="N72" s="22" t="str">
+      <c r="N72" s="20" t="str">
         <f aca="true">IF(B72="","",IF(AND(M72&lt;&gt;"",M72&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K72&lt;&gt;"",TODAY()-K72&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4308,7 +4329,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B73" s="19"/>
       <c r="C73" s="15"/>
@@ -4322,7 +4343,7 @@
       <c r="K73" s="17"/>
       <c r="L73" s="19"/>
       <c r="M73" s="17"/>
-      <c r="N73" s="22" t="str">
+      <c r="N73" s="20" t="str">
         <f aca="true">IF(B73="","",IF(AND(M73&lt;&gt;"",M73&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K73&lt;&gt;"",TODAY()-K73&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4330,7 +4351,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B74" s="19"/>
       <c r="C74" s="15"/>
@@ -4344,7 +4365,7 @@
       <c r="K74" s="17"/>
       <c r="L74" s="19"/>
       <c r="M74" s="17"/>
-      <c r="N74" s="22" t="str">
+      <c r="N74" s="20" t="str">
         <f aca="true">IF(B74="","",IF(AND(M74&lt;&gt;"",M74&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K74&lt;&gt;"",TODAY()-K74&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4352,7 +4373,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B75" s="19"/>
       <c r="C75" s="15"/>
@@ -4366,7 +4387,7 @@
       <c r="K75" s="17"/>
       <c r="L75" s="19"/>
       <c r="M75" s="17"/>
-      <c r="N75" s="22" t="str">
+      <c r="N75" s="20" t="str">
         <f aca="true">IF(B75="","",IF(AND(M75&lt;&gt;"",M75&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K75&lt;&gt;"",TODAY()-K75&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4374,7 +4395,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B76" s="19"/>
       <c r="C76" s="15"/>
@@ -4388,7 +4409,7 @@
       <c r="K76" s="17"/>
       <c r="L76" s="19"/>
       <c r="M76" s="17"/>
-      <c r="N76" s="22" t="str">
+      <c r="N76" s="20" t="str">
         <f aca="true">IF(B76="","",IF(AND(M76&lt;&gt;"",M76&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K76&lt;&gt;"",TODAY()-K76&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4396,7 +4417,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B77" s="19"/>
       <c r="C77" s="15"/>
@@ -4410,7 +4431,7 @@
       <c r="K77" s="17"/>
       <c r="L77" s="19"/>
       <c r="M77" s="17"/>
-      <c r="N77" s="22" t="str">
+      <c r="N77" s="20" t="str">
         <f aca="true">IF(B77="","",IF(AND(M77&lt;&gt;"",M77&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K77&lt;&gt;"",TODAY()-K77&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4418,7 +4439,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B78" s="19"/>
       <c r="C78" s="15"/>
@@ -4432,7 +4453,7 @@
       <c r="K78" s="17"/>
       <c r="L78" s="19"/>
       <c r="M78" s="17"/>
-      <c r="N78" s="22" t="str">
+      <c r="N78" s="20" t="str">
         <f aca="true">IF(B78="","",IF(AND(M78&lt;&gt;"",M78&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K78&lt;&gt;"",TODAY()-K78&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4440,7 +4461,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B79" s="19"/>
       <c r="C79" s="15"/>
@@ -4454,7 +4475,7 @@
       <c r="K79" s="17"/>
       <c r="L79" s="19"/>
       <c r="M79" s="17"/>
-      <c r="N79" s="22" t="str">
+      <c r="N79" s="20" t="str">
         <f aca="true">IF(B79="","",IF(AND(M79&lt;&gt;"",M79&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K79&lt;&gt;"",TODAY()-K79&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4462,7 +4483,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B80" s="19"/>
       <c r="C80" s="15"/>
@@ -4476,7 +4497,7 @@
       <c r="K80" s="17"/>
       <c r="L80" s="19"/>
       <c r="M80" s="17"/>
-      <c r="N80" s="22" t="str">
+      <c r="N80" s="20" t="str">
         <f aca="true">IF(B80="","",IF(AND(M80&lt;&gt;"",M80&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K80&lt;&gt;"",TODAY()-K80&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4484,7 +4505,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B81" s="19"/>
       <c r="C81" s="15"/>
@@ -4498,7 +4519,7 @@
       <c r="K81" s="17"/>
       <c r="L81" s="19"/>
       <c r="M81" s="17"/>
-      <c r="N81" s="22" t="str">
+      <c r="N81" s="20" t="str">
         <f aca="true">IF(B81="","",IF(AND(M81&lt;&gt;"",M81&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K81&lt;&gt;"",TODAY()-K81&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4506,7 +4527,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B82" s="19"/>
       <c r="C82" s="15"/>
@@ -4520,7 +4541,7 @@
       <c r="K82" s="17"/>
       <c r="L82" s="19"/>
       <c r="M82" s="17"/>
-      <c r="N82" s="22" t="str">
+      <c r="N82" s="20" t="str">
         <f aca="true">IF(B82="","",IF(AND(M82&lt;&gt;"",M82&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K82&lt;&gt;"",TODAY()-K82&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4528,7 +4549,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B83" s="19"/>
       <c r="C83" s="15"/>
@@ -4542,7 +4563,7 @@
       <c r="K83" s="17"/>
       <c r="L83" s="19"/>
       <c r="M83" s="17"/>
-      <c r="N83" s="22" t="str">
+      <c r="N83" s="20" t="str">
         <f aca="true">IF(B83="","",IF(AND(M83&lt;&gt;"",M83&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K83&lt;&gt;"",TODAY()-K83&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4550,7 +4571,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B84" s="19"/>
       <c r="C84" s="15"/>
@@ -4564,7 +4585,7 @@
       <c r="K84" s="17"/>
       <c r="L84" s="19"/>
       <c r="M84" s="17"/>
-      <c r="N84" s="22" t="str">
+      <c r="N84" s="20" t="str">
         <f aca="true">IF(B84="","",IF(AND(M84&lt;&gt;"",M84&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K84&lt;&gt;"",TODAY()-K84&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4572,7 +4593,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B85" s="19"/>
       <c r="C85" s="15"/>
@@ -4586,7 +4607,7 @@
       <c r="K85" s="17"/>
       <c r="L85" s="19"/>
       <c r="M85" s="17"/>
-      <c r="N85" s="22" t="str">
+      <c r="N85" s="20" t="str">
         <f aca="true">IF(B85="","",IF(AND(M85&lt;&gt;"",M85&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K85&lt;&gt;"",TODAY()-K85&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4594,7 +4615,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B86" s="19"/>
       <c r="C86" s="15"/>
@@ -4608,7 +4629,7 @@
       <c r="K86" s="17"/>
       <c r="L86" s="19"/>
       <c r="M86" s="17"/>
-      <c r="N86" s="22" t="str">
+      <c r="N86" s="20" t="str">
         <f aca="true">IF(B86="","",IF(AND(M86&lt;&gt;"",M86&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K86&lt;&gt;"",TODAY()-K86&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4616,7 +4637,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B87" s="19"/>
       <c r="C87" s="15"/>
@@ -4630,7 +4651,7 @@
       <c r="K87" s="17"/>
       <c r="L87" s="19"/>
       <c r="M87" s="17"/>
-      <c r="N87" s="22" t="str">
+      <c r="N87" s="20" t="str">
         <f aca="true">IF(B87="","",IF(AND(M87&lt;&gt;"",M87&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K87&lt;&gt;"",TODAY()-K87&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4638,7 +4659,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B88" s="19"/>
       <c r="C88" s="15"/>
@@ -4652,7 +4673,7 @@
       <c r="K88" s="17"/>
       <c r="L88" s="19"/>
       <c r="M88" s="17"/>
-      <c r="N88" s="22" t="str">
+      <c r="N88" s="20" t="str">
         <f aca="true">IF(B88="","",IF(AND(M88&lt;&gt;"",M88&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K88&lt;&gt;"",TODAY()-K88&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4660,7 +4681,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B89" s="19"/>
       <c r="C89" s="15"/>
@@ -4674,7 +4695,7 @@
       <c r="K89" s="17"/>
       <c r="L89" s="19"/>
       <c r="M89" s="17"/>
-      <c r="N89" s="22" t="str">
+      <c r="N89" s="20" t="str">
         <f aca="true">IF(B89="","",IF(AND(M89&lt;&gt;"",M89&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K89&lt;&gt;"",TODAY()-K89&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4682,7 +4703,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B90" s="19"/>
       <c r="C90" s="15"/>
@@ -4696,7 +4717,7 @@
       <c r="K90" s="17"/>
       <c r="L90" s="19"/>
       <c r="M90" s="17"/>
-      <c r="N90" s="22" t="str">
+      <c r="N90" s="20" t="str">
         <f aca="true">IF(B90="","",IF(AND(M90&lt;&gt;"",M90&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K90&lt;&gt;"",TODAY()-K90&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4704,7 +4725,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B91" s="19"/>
       <c r="C91" s="15"/>
@@ -4718,7 +4739,7 @@
       <c r="K91" s="17"/>
       <c r="L91" s="19"/>
       <c r="M91" s="17"/>
-      <c r="N91" s="22" t="str">
+      <c r="N91" s="20" t="str">
         <f aca="true">IF(B91="","",IF(AND(M91&lt;&gt;"",M91&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K91&lt;&gt;"",TODAY()-K91&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4726,7 +4747,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B92" s="19"/>
       <c r="C92" s="15"/>
@@ -4740,7 +4761,7 @@
       <c r="K92" s="17"/>
       <c r="L92" s="19"/>
       <c r="M92" s="17"/>
-      <c r="N92" s="22" t="str">
+      <c r="N92" s="20" t="str">
         <f aca="true">IF(B92="","",IF(AND(M92&lt;&gt;"",M92&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K92&lt;&gt;"",TODAY()-K92&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4748,7 +4769,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B93" s="19"/>
       <c r="C93" s="15"/>
@@ -4762,7 +4783,7 @@
       <c r="K93" s="17"/>
       <c r="L93" s="19"/>
       <c r="M93" s="17"/>
-      <c r="N93" s="22" t="str">
+      <c r="N93" s="20" t="str">
         <f aca="true">IF(B93="","",IF(AND(M93&lt;&gt;"",M93&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K93&lt;&gt;"",TODAY()-K93&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4770,7 +4791,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B94" s="19"/>
       <c r="C94" s="15"/>
@@ -4784,7 +4805,7 @@
       <c r="K94" s="17"/>
       <c r="L94" s="19"/>
       <c r="M94" s="17"/>
-      <c r="N94" s="22" t="str">
+      <c r="N94" s="20" t="str">
         <f aca="true">IF(B94="","",IF(AND(M94&lt;&gt;"",M94&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K94&lt;&gt;"",TODAY()-K94&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4792,7 +4813,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B95" s="19"/>
       <c r="C95" s="15"/>
@@ -4806,7 +4827,7 @@
       <c r="K95" s="17"/>
       <c r="L95" s="19"/>
       <c r="M95" s="17"/>
-      <c r="N95" s="22" t="str">
+      <c r="N95" s="20" t="str">
         <f aca="true">IF(B95="","",IF(AND(M95&lt;&gt;"",M95&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K95&lt;&gt;"",TODAY()-K95&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4814,7 +4835,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B96" s="19"/>
       <c r="C96" s="15"/>
@@ -4828,7 +4849,7 @@
       <c r="K96" s="17"/>
       <c r="L96" s="19"/>
       <c r="M96" s="17"/>
-      <c r="N96" s="22" t="str">
+      <c r="N96" s="20" t="str">
         <f aca="true">IF(B96="","",IF(AND(M96&lt;&gt;"",M96&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K96&lt;&gt;"",TODAY()-K96&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4836,7 +4857,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B97" s="19"/>
       <c r="C97" s="15"/>
@@ -4850,7 +4871,7 @@
       <c r="K97" s="17"/>
       <c r="L97" s="19"/>
       <c r="M97" s="17"/>
-      <c r="N97" s="22" t="str">
+      <c r="N97" s="20" t="str">
         <f aca="true">IF(B97="","",IF(AND(M97&lt;&gt;"",M97&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K97&lt;&gt;"",TODAY()-K97&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4858,7 +4879,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B98" s="19"/>
       <c r="C98" s="15"/>
@@ -4872,7 +4893,7 @@
       <c r="K98" s="17"/>
       <c r="L98" s="19"/>
       <c r="M98" s="17"/>
-      <c r="N98" s="22" t="str">
+      <c r="N98" s="20" t="str">
         <f aca="true">IF(B98="","",IF(AND(M98&lt;&gt;"",M98&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K98&lt;&gt;"",TODAY()-K98&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4880,7 +4901,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B99" s="19"/>
       <c r="C99" s="15"/>
@@ -4894,7 +4915,7 @@
       <c r="K99" s="17"/>
       <c r="L99" s="19"/>
       <c r="M99" s="17"/>
-      <c r="N99" s="22" t="str">
+      <c r="N99" s="20" t="str">
         <f aca="true">IF(B99="","",IF(AND(M99&lt;&gt;"",M99&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K99&lt;&gt;"",TODAY()-K99&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4902,7 +4923,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B100" s="19"/>
       <c r="C100" s="15"/>
@@ -4916,7 +4937,7 @@
       <c r="K100" s="17"/>
       <c r="L100" s="19"/>
       <c r="M100" s="17"/>
-      <c r="N100" s="22" t="str">
+      <c r="N100" s="20" t="str">
         <f aca="true">IF(B100="","",IF(AND(M100&lt;&gt;"",M100&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K100&lt;&gt;"",TODAY()-K100&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4924,7 +4945,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B101" s="19"/>
       <c r="C101" s="15"/>
@@ -4938,7 +4959,7 @@
       <c r="K101" s="17"/>
       <c r="L101" s="19"/>
       <c r="M101" s="17"/>
-      <c r="N101" s="22" t="str">
+      <c r="N101" s="20" t="str">
         <f aca="true">IF(B101="","",IF(AND(M101&lt;&gt;"",M101&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K101&lt;&gt;"",TODAY()-K101&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4946,7 +4967,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B102" s="19"/>
       <c r="C102" s="15"/>
@@ -4960,7 +4981,7 @@
       <c r="K102" s="17"/>
       <c r="L102" s="19"/>
       <c r="M102" s="17"/>
-      <c r="N102" s="22" t="str">
+      <c r="N102" s="20" t="str">
         <f aca="true">IF(B102="","",IF(AND(M102&lt;&gt;"",M102&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K102&lt;&gt;"",TODAY()-K102&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4968,7 +4989,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="7" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B103" s="19"/>
       <c r="C103" s="15"/>
@@ -4982,7 +5003,7 @@
       <c r="K103" s="17"/>
       <c r="L103" s="19"/>
       <c r="M103" s="17"/>
-      <c r="N103" s="22" t="str">
+      <c r="N103" s="20" t="str">
         <f aca="true">IF(B103="","",IF(AND(M103&lt;&gt;"",M103&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K103&lt;&gt;"",TODAY()-K103&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
@@ -4990,7 +5011,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B104" s="19"/>
       <c r="C104" s="15"/>
@@ -5004,62 +5025,40 @@
       <c r="K104" s="17"/>
       <c r="L104" s="19"/>
       <c r="M104" s="17"/>
-      <c r="N104" s="22" t="str">
+      <c r="N104" s="20" t="str">
         <f aca="true">IF(B104="","",IF(AND(M104&lt;&gt;"",M104&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K104&lt;&gt;"",TODAY()-K104&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
         <v/>
       </c>
       <c r="O104" s="19"/>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="B105" s="19"/>
-      <c r="C105" s="15"/>
-      <c r="D105" s="19"/>
-      <c r="E105" s="19"/>
-      <c r="F105" s="19"/>
-      <c r="G105" s="19"/>
-      <c r="H105" s="15"/>
-      <c r="I105" s="15"/>
-      <c r="J105" s="15"/>
-      <c r="K105" s="17"/>
-      <c r="L105" s="19"/>
-      <c r="M105" s="17"/>
-      <c r="N105" s="22" t="str">
-        <f aca="true">IF(B105="","",IF(AND(M105&lt;&gt;"",M105&lt;TODAY()),"Quá hạn việc tiếp theo",IF(AND(K105&lt;&gt;"",TODAY()-K105&gt;30),"Hơn 30 ngày chưa liên hệ","")))</f>
-        <v/>
-      </c>
-      <c r="O105" s="19"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:O105"/>
+  <autoFilter ref="A4:O104"/>
   <mergeCells count="1">
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="N6:N105">
+  <conditionalFormatting sqref="N5:N104">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>ISNUMBER(SEARCH("quá hạn",N6))</formula>
+      <formula>ISNUMBER(SEARCH("quá hạn",N5))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C5:C105" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C5:C104" type="list">
       <formula1>"A. Technology,B. Channel / SI,C. Domain consultant,D. Ecosystem"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D5:D105" type="list">
+    <dataValidation allowBlank="true" error="Giá trị này không nằm trong danh sách. Chọn tiếp tục nếu muốn nhập nhiều ngành, cách nhau bằng dấu chấm phẩy." errorStyle="warning" errorTitle="Ngành" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D5:D104" type="list">
       <formula1>"BFSI,Chính phủ,Y tế,Bán lẻ,Sản xuất,Logistics,Truyền thông,Giáo dục"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H5:H105" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H5:H104" type="list">
       <formula1>"1. Tìm,2. Tiếp cận,3. Thẩm định,4. Ký,5. Onboarding,6. Kích hoạt,7. Tạo giá trị,8. Đánh giá"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I5:I105" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I5:I104" type="list">
       <formula1>"Explorer,Certified,Strategic"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Nhập điểm từ 1 đến 5" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J5:J105" type="whole">
+    <dataValidation allowBlank="true" error="Nhập điểm từ 1 đến 5" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J5:J104" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
@@ -5095,12 +5094,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -5114,42 +5113,42 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C5" s="15" t="s">
         <v>134</v>
@@ -5166,15 +5165,15 @@
         <v/>
       </c>
       <c r="J5" s="19" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>188</v>
+        <v>171</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>134</v>
@@ -5191,15 +5190,15 @@
         <v/>
       </c>
       <c r="J6" s="19" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>134</v>
@@ -5216,15 +5215,15 @@
         <v/>
       </c>
       <c r="J7" s="19" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>134</v>
@@ -5241,15 +5240,15 @@
         <v/>
       </c>
       <c r="J8" s="19" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>134</v>
@@ -5266,15 +5265,15 @@
         <v/>
       </c>
       <c r="J9" s="19" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>134</v>
@@ -5291,23 +5290,33 @@
         <v/>
       </c>
       <c r="J10" s="19" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="15"/>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
+        <v>202</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>134</v>
+      </c>
       <c r="D11" s="17"/>
       <c r="E11" s="17"/>
       <c r="F11" s="19"/>
       <c r="G11" s="19"/>
-      <c r="H11" s="15"/>
+      <c r="H11" s="15" t="s">
+        <v>134</v>
+      </c>
       <c r="I11" s="18" t="str">
         <f aca="true">IF(E11="","",IF(E11&lt;TODAY(),"Hết hạn",IF(E11-TODAY()&lt;=60,"Sắp hết hạn","Còn hiệu lực")))</f>
         <v/>
       </c>
-      <c r="J11" s="19"/>
+      <c r="J11" s="19" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19"/>
@@ -5711,32 +5720,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>60</v>
@@ -5744,10 +5753,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>7</v>
@@ -5765,10 +5774,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="C6" s="15" t="n">
         <v>7</v>
@@ -5786,10 +5795,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="C7" s="15" t="n">
         <v>30</v>
@@ -5807,10 +5816,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C8" s="15" t="n">
         <v>90</v>
@@ -5828,10 +5837,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C9" s="15" t="n">
         <v>90</v>
@@ -5849,10 +5858,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C10" s="15" t="n">
         <v>90</v>

</xml_diff>